<commit_message>
Fix generic filler descriptions in Units 5-6 coding questions
Same fix as Units 2-4: rewrote the 10 placeholder descriptions in each
unit with a real scenario and explicit logic, verified against existing
solutions/test cases.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/Question Bank/Coding Questions/Unit 5 - Strings/Unit 5 - Strings - Coding Questions.xlsx
+++ b/content/Question Bank/Coding Questions/Unit 5 - Strings/Unit 5 - Strings - Coding Questions.xlsx
@@ -1887,18 +1887,18 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A ticketing system generates short boarding codes by taking the first three characters of a passenger's name.
-Read a line of text and print its first three characters, in order. If the text has fewer than three characters, print the text exactly as it is (there aren't enough characters to trim).
+          <t>An airline's booking system generates a short destination code for every ticket by taking just the first three letters of the city name typed in by the check-in agent.
+Write a program that reads a city name and prints only its first three characters. If the name has fewer than three characters, print the whole name.
 ### Input Format
-- Line 1: Text
+- Line 1: City name
 ### Output Format
 ```
 Pyt
 ```
 ### Example Walkthrough
-In the sample, the text is `Python`. Its first three characters are `P`, `y`, and `t`, so the program prints `Pyt`.
+In the sample, the city name is `Python`. Taking the first three characters gives `Pyt`, which the program prints.
 ### Constraints
-- The text may contain fewer than three characters, in which case the entire text is printed.
+- The input is a valid line of text with no leading or trailing spaces.
 - Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
@@ -2044,18 +2044,18 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A sentence-checking tool in a writing app flags whether a line ends with proper punctuation.
-Read a line of text. If the last character of the text is a period (`.`), print `Yes`; otherwise print `No`.
+          <t>A grammar checker flags whether a sentence a student submits ends with proper punctuation, specifically a full stop.
+Write a program that reads a line of text and prints `Yes` if it ends with a period (`.`), and `No` otherwise.
 ### Input Format
-- Line 1: Text
+- Line 1: A sentence
 ### Output Format
 ```
 Yes
 ```
 ### Example Walkthrough
-In the sample, the text is `Hello.`. Its last character is `.`, so the program prints `Yes`.
+In the sample, the text is `Hello.`. Since the last character is a period, the program prints `Yes`. The text `Hello` (no period) would print `No`.
 ### Constraints
-- The check looks only at the very last character of the text.
+- The input is a valid line of text with no leading or trailing spaces.
 - Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
@@ -3667,8 +3667,8 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A sign-up form on ByteXL's portal wants to store usernames in a clean, consistent form regardless of how a user typed them.
-Read a line containing a username. Remove any leading and trailing spaces, convert all letters to lower case, and print the result.
+          <t>A signup form normalizes every username before storing it in the database, so `  Asha  ` and `asha` are treated as the same account: stray spaces at the ends are trimmed and every letter is converted to lower case.
+Write a program that reads a username, removes any leading or trailing spaces, converts it to lower case, and prints the result.
 ### Input Format
 - Line 1: Username
 ### Output Format
@@ -3676,9 +3676,9 @@
 asha
 ```
 ### Example Walkthrough
-In the sample, the input is `  Asha  ` (with extra spaces around it). Removing the leading and trailing spaces gives `Asha`, and converting it to lower case gives `asha`, which the program prints.
+In the sample, the input is `  Asha  `. Trimming the spaces gives `Asha`, and converting to lower case gives `asha`, which the program prints.
 ### Constraints
-- Only leading and trailing spaces are removed; spaces between words, if any, are kept.
+- The input is a valid line of text.
 - Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
@@ -3823,18 +3823,18 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A URL-building tool needs to turn a spoken phrase into a hyphen-separated slug fragment.
-Read a line of one or more words separated by spaces. Join the words together using a hyphen (`-`) between each pair, and print the result.
+          <t>A photo-sharing app turns a caption typed with spaces into a single hashtag by joining the words together with hyphens instead of spaces.
+Write a program that reads a line of words separated by spaces and prints them joined together with a single hyphen (`-`) between each pair of words.
 ### Input Format
-- Line 1: Words
+- Line 1: Words separated by spaces
 ### Output Format
 ```
 hello-world
 ```
 ### Example Walkthrough
-In the sample, the input is `hello world`, which splits into the words `hello` and `world`. Joining them with a hyphen gives `hello-world`, which the program prints.
+In the sample, the input is `hello world`. Splitting it gives the words `hello` and `world`, and joining them with a hyphen gives `hello-world`, which the program prints.
 ### Constraints
-- Words may be separated by one or more spaces in the input, but the output uses exactly one hyphen between each pair of words.
+- The input is a valid line of text with at least one word.
 - Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
@@ -5287,18 +5287,18 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>A word game removes the first and last letter of a word to create a new puzzle clue.
-Read a line of text. Print the text with its first and last character removed, keeping everything in between. If the text has two or fewer characters, nothing remains, so print an empty line.
+          <t>A text editor's "trim edges" feature strips away the very first and last character of any word a user selects, leaving just the middle portion behind.
+Write a program that reads a word and prints it with its first and last characters removed. If the word has one or two characters, print an empty line.
 ### Input Format
-- Line 1: Text
+- Line 1: A word
 ### Output Format
 ```
 ytho
 ```
 ### Example Walkthrough
-In the sample, the text is `Python`. Removing the first character `P` and the last character `n` leaves `ytho`, which the program prints.
+In the sample, the word is `Python`. Removing the first character (`P`) and the last character (`n`) leaves `ytho`, which the program prints.
 ### Constraints
-- If the text has one or two characters, the result is empty and the program prints a blank line.
+- The input is a valid word with no spaces.
 - Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
@@ -5434,19 +5434,19 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A study app highlights how often a target word appears in a sentence to help students spot repetition.
-Read a sentence, then a word. Split the sentence into words wherever there is a space, and count how many of those words are exactly equal to the given word (matching is case-sensitive). Print the count.
+          <t>An analytics tool checks how many times a specific keyword appears among the words of a sentence a user has typed, to measure keyword repetition. The match must be an exact, case-sensitive whole word, not a substring.
+Write a program that reads a sentence on one line and a target word on the next line, then prints how many of the sentence's space-separated words exactly match the target word.
 ### Input Format
-- Line 1: Sentence
-- Line 2: Word
+- Line 1: A sentence (words separated by spaces)
+- Line 2: The target word
 ### Output Format
 ```
 2
 ```
 ### Example Walkthrough
-In the sample, the sentence is `cat dog cat` and the word is `cat`. Splitting the sentence gives the words `cat`, `dog`, `cat`, and exactly `2` of them equal `cat`, so the program prints `2`.
+In the sample, the sentence is `cat dog cat` and the target word is `cat`. Splitting the sentence into words gives `cat`, `dog`, and `cat`, of which two exactly match `cat`, so the program prints `2`.
 ### Constraints
-- The match is case-sensitive and compares whole words only, not substrings.
+- The inputs are valid lines of text with no leading or trailing spaces.
 - Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
@@ -5598,18 +5598,18 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A privacy feature in an email client hides the username part of an address before showing it on screen.
-Read an email address containing exactly one `@`. Replace every character before the `@` with an asterisk (`*`), keeping the same number of characters, then print the masked name followed by `@` and the domain part unchanged.
+          <t>A public leaderboard shows partial email addresses for privacy: the part before the `@` is replaced with the same number of asterisks, while the domain after the `@` stays visible.
+Write a program that reads an email address and prints it with the part before the `@` replaced by that many asterisks, keeping the `@` and everything after it unchanged.
 ### Input Format
-- Line 1: Email
+- Line 1: An email address in the form `name@domain`
 ### Output Format
 ```
 ****@mail.com
 ```
 ### Example Walkthrough
-In the sample, the email is `asha@mail.com`. The part before `@` is `asha`, which has 4 characters, so it becomes `****`. The domain `mail.com` after the `@` stays unchanged, so the program prints `****@mail.com`.
+In the sample, the email is `asha@mail.com`. The part before `@` is `asha`, which has 4 characters, so it becomes `****`, and the program prints `****@mail.com`.
 ### Constraints
-- The email contains exactly one `@` symbol separating the name from the domain.
+- The input is a valid email address containing exactly one `@`.
 - Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
@@ -7093,18 +7093,18 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>A simple file-compression demo shrinks text by replacing repeated runs of the same character with the character and its count.
-Read a line of text. Scan through it and group consecutive occurrences of the same character into runs. For each run, print the character followed by how many times it repeats, one run after another with no separators.
+          <t>A simple image tool draws pixel rows as sequences of colored strokes, and compresses each row for storage by writing each repeated color once followed by how many pixels in a row had that color.
+Write a program that reads a string and prints its run-length encoding: each maximal run of the same consecutive character replaced by that character followed by the count of how many times it repeats, with no separators between runs.
 ### Input Format
-- Line 1: Text
+- Line 1: A string with no spaces
 ### Output Format
 ```
 a3b2
 ```
 ### Example Walkthrough
-In the sample, the text is `aaabb`. It has a run of three `a`s followed by a run of two `b`s, so the program prints `a3b2`.
+In the sample, the string is `aaabb`. The first run is `a` repeated 3 times (`a3`), followed by `b` repeated 2 times (`b2`), so the program prints `a3b2`.
 ### Constraints
-- Every character in the input, including digits, is treated the same way when grouping runs.
+- The input is a valid non-empty string with no spaces.
 - Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
@@ -7254,18 +7254,18 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>A puzzle app reverses the order of words in a sentence while keeping each word itself unchanged.
-Read a line of text. Split it into words wherever there is a space, reverse the order of the words, and print them back joined by single spaces.
+          <t>A teleprompter app has a "word-order drill" mode for practicing sentences backwards: it takes a sentence and reads the words out in reverse order, without spelling any individual word backwards.
+Write a program that reads a sentence and prints its words in reverse order, separated by single spaces.
 ### Input Format
-- Line 1: Text
+- Line 1: A sentence (words separated by spaces)
 ### Output Format
 ```
 three two one
 ```
 ### Example Walkthrough
-In the sample, the input is `one two three`, which splits into the words `one`, `two`, `three`. Reversing their order gives `three`, `two`, `one`, so the program prints `three two one`.
+In the sample, the sentence is `one two three`. Splitting it into words gives `one`, `two`, `three`, and reversing their order gives `three`, `two`, `one`, so the program prints `three two one`.
 ### Constraints
-- Only the order of the words is reversed; the letters within each word stay the same.
+- The input is a valid line of text with at least one word.
 - Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>
@@ -7410,19 +7410,19 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>A word-puzzle app checks whether two phrases are anagrams of each other, ignoring case and spaces.
-Read two lines of text. Convert both to lower case and remove all spaces from each. If the sorted letters of the first line match the sorted letters of the second line exactly, print `Yes`; otherwise print `No`.
+          <t>A word puzzle game checks whether a player's submitted word is an anagram of the target word — made of exactly the same letters rearranged — ignoring letter case and any spaces.
+Write a program that reads two words on separate lines, ignores case and spaces in both, and prints `Yes` if they are anagrams of each other, and `No` otherwise.
 ### Input Format
-- Line 1: First
-- Line 2: Second
+- Line 1: First word
+- Line 2: Second word
 ### Output Format
 ```
 Yes
 ```
 ### Example Walkthrough
-In the sample, the first line is `listen` and the second is `silent`. Neither has spaces, and after converting to lower case and sorting their letters, both become `eilnst`, so the program prints `Yes`.
+In the sample, the words are `listen` and `silent`. Both contain exactly the same letters, just rearranged, so the program prints `Yes`.
 ### Constraints
-- Comparison ignores letter case and spaces but considers every other character, including punctuation and digits.
+- The inputs are valid lines of text.
 - Every value must be printed exactly as shown in the output format, with no extra text added or removed.</t>
         </is>
       </c>

</xml_diff>